<commit_message>
feat(F-NAR-019): ATOM-EMO.GES.001-01 Stop près du banc
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.GES.001-01.xlsx
+++ b/stories/arbres/ATOM-EMO.GES.001-01.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>parc</t>
+          <t>parc, balançoire, chaîne, siège de caoutchouc, fer, herbe, poussière, abeille, seau</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Victorina, Chouchou, maman</t>
+          <t>Amir, Nino, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Au parc, le câlin de Chouchou est trop fort. Victorina dit stop. Elle recule. Elle va vers maman, l'adulte du banc.</t>
+          <t>La chaîne de la balançoire tinte au soleil. Sur le fer, un éclat de balançoire luit. Amir veut jouer, maintenant. Nino serre trop. Poitrine coincée. Sourire parti. Papa s'accroupit. Amir dit stop, recule d'un pas. Merci vécu. Nino se colle trop près du siège. Amir refuse de foncer. Un éclat de balançoire tient sur le fer.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Le banc du parc est encore chaud. Le bois sent le soleil. L'herbe coupée sent fort. Une chaîne de balançoire tinte. Une feuille sèche tourne sur le chemin. Un oiseau crie tout près, puis plus. Je suis sur le banc, Victorina. Tu joues près du bac à sable ? Oui, maman. En ce moment, Victorina est près du bac. Le sable est tiède sous les doigts. Elle fait un petit tas, tout rond. Je te vois, Victorina. Le banc est juste ici. Mon tas est rond. Il est bien rond, oui. Chouchou arrive, tout content. Il veut un câlin. Le câlin est trop fort. Victorina sent sa poitrine coincée. Ses épaules montent. Je n'aime pas. C'est trop. Stop. Elle recule d'un pas. Elle peut s'éloigner. Elle s'éloigne vers le banc. Maman est l'adulte sur le banc. Victorina va vers maman. C'était trop. Je t'écoute. Tu as dit stop. Tu t'es éloignée. Tu es venue vers moi. Victorina pose sa main dans la main de maman. Souffle un peu. Victorina souffle. Ses épaules descendent. Dire stop, c'est permis. On s'éloigne. On va vers un adulte. Stop. Puis le banc. Bravo, Victorina. Tu as les épaules plus douces, maintenant ? Oui, maman. Chouchou reste près du bac. Il joue avec le sable. Victorina reste près du banc. Tu veux rester assise ici ? Oui. Près de toi. On regarde la feuille, ensemble. La feuille sèche a arrêté de tourner. Le banc est chaud sous les jambes. Je me suis éloignée. Oui. Vers un adulte. C'est le bon geste.</t>
+          <t>La chaîne de la balançoire tinte au soleil. Elle tinte, papa. Tu l'entends, la chaîne ? Oui, papa. Le siège sent le caoutchouc chaud. Il est chaud, Amir ? Un peu, maman. Papa tapote le fer du siège. Toc, toc, sur le métal. Tu entends le fer, Amir ? Oui, il sonne. Maman pose la main sur le siège. Le caoutchouc est tiède, un peu rêche. Sur le fer, un éclat de balançoire luit. Il brille, maman. Tu le vois, sur le fer ? Oui, un petit point. Le soleil le touche. Un rayon glisse entre les chaînes. La poussière dore, près des pieds. Elle chatouille le pantalon. Elle est chaude. Tu t'assois, Amir ? Un peu. Une abeille visite une chaussure. Elle fait un petit bzz. Elle part. L'abeille a fini. L'herbe du parc sent le soleil. Ça sent l'herbe, maman. Tu la sens, l'herbe chaude ? Oui, maman. En ce moment, Amir prend la chaîne. Je veux jouer, maintenant ! Tout de suite ? Oui, papa. Les mains serrent le fer tiède. Tu pousses le siège ? Oui, maman. Nino arrive près de la balançoire. Il ouvre les bras trop vite. Un câlin ! Tu viens, Nino ? Oui. Nino serre Amir contre lui. Le câlin colle trop fort. Oh. Je te tiens. Amir sent sa poitrine coincée. Le sourire d'Amir disparaît. Dans sa poitrine, ça se bouscule. L'envie et la peur se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Nino, Amir ? Oui, papa. Tes mains sont chaudes, Amir ? Un peu, maman. L'éclat de balançoire tremble, puis tient.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Le banc du parc est encore chaud. Le bois sent le soleil. L'herbe coupée sent fort. Une chaîne de balançoire tinte. Une feuille sèche tourne sur le chemin. Un oiseau crie tout près, puis plus. Je suis sur le banc, Victorina. Tu joues près du bac à sable ? Oui, maman. En ce moment, Victorina est près du bac. Le sable est tiède sous les doigts. Elle fait un petit tas, tout rond. Je te vois, Victorina. Le banc est juste ici. Mon tas est rond. Il est bien rond, oui. Chouchou arrive, tout content. Il veut un câlin. Le câlin est trop fort. Victorina sent sa poitrine coincée. Ses épaules montent. Je n'aime pas. C'est trop. Stop. Elle recule d'un pas. Elle peut s'éloigner. Elle s'éloigne vers le banc. Maman est l'adulte sur le banc. Victorina va vers maman. C'était trop. Je t'écoute. Tu as dit stop. Tu t'es éloignée. Tu es venue vers moi. Victorina pose sa main dans la main de maman. Souffle un peu. Victorina souffle. Ses épaules descendent. Dire stop, c'est permis. On s'éloigne. On va vers un adulte. Stop. Puis le banc. Bravo, Victorina. Tu as les épaules plus douces, maintenant ? Oui, maman. Chouchou reste près du bac. Il joue avec le sable. Victorina reste près du banc. Tu veux rester assise ici ? Oui. Près de toi. On regarde la feuille, ensemble. La feuille sèche a arrêté de tourner. Le banc est chaud sous les jambes. Je me suis éloignée. Oui. Vers un adulte. C'est le bon geste.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La chaîne de la balançoire tinte au soleil. Elle tinte, papa. Tu l'entends, la chaîne ? Oui, papa. Le siège sent le caoutchouc chaud. Il est chaud, Amir ? Un peu, maman. Papa tapote le fer du siège. Toc, toc, sur le métal. Tu entends le fer, Amir ? Oui, il sonne. Maman pose la main sur le siège. Le caoutchouc est tiède, un peu rêche. Sur le fer, un &lt;emphasis level="moderate"&gt;éclat de balançoire&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, sur le fer ? Oui, un petit point. Le soleil le touche. Un rayon glisse entre les chaînes. La poussière dore, près des pieds. Elle chatouille le pantalon. Elle est chaude. Tu t'assois, Amir ? Un peu. Une abeille visite une chaussure. Elle fait un petit bzz. Elle part. L'abeille a fini. L'herbe du parc sent le soleil. Ça sent l'herbe, maman. Tu la sens, l'herbe chaude ? Oui, maman. En ce moment, Amir prend la chaîne. Je veux jouer, maintenant ! Tout de suite ? Oui, papa. Les mains serrent le fer tiède. Tu pousses le siège ? Oui, maman. Nino arrive près de la balançoire. Il ouvre les bras trop vite. Un câlin ! Tu viens, Nino ? Oui. Nino serre Amir contre lui. Le câlin colle trop fort. Oh. Je te tiens. Amir sent sa poitrine coincée. Le sourire d'Amir disparaît. Dans sa poitrine, ça se bouscule. L'envie et la peur se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Nino, Amir ? Oui, papa. Tes mains sont chaudes, Amir ? Un peu, maman. L'éclat de balançoire tremble, puis tient.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Adam joue au parc. Un camarade le serre trop fort. Adam sent sa poitrine coincée. Il dit : je n'aime pas. C'est trop. Adam dit : &lt;emphasis&gt;stop&lt;/emphasis&gt;. Il recule d'un pas. Il peut s'éloigner. Il s'éloigne vers le banc. Maman est l'adulte sur le banc. Adam va vers maman. Il dit : c'était trop. Maman l'écoute. Adam pose sa main dans la main de maman. Il souffle. Ses épaules descendent. Dire stop, c'est permis. On s'éloigne. On va vers un adulte.&lt;/slow&gt; [pause]</t>
+          <t>La chaîne de la balançoire tinte au soleil. Elle tinte, papa. Tu l'entends, la chaîne ? Oui, papa. Le siège sent le caoutchouc chaud. Il est chaud, Amir ? Un peu, maman. Papa tapote le fer du siège. Toc, toc, sur le métal. Tu entends le fer, Amir ? Oui, il sonne. Maman pose la main sur le siège. Le caoutchouc est tiède, un peu rêche. Sur le fer, un &lt;emphasis&gt;éclat de balançoire&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, sur le fer ? Oui, un petit point. Le soleil le touche. Un rayon glisse entre les chaînes. La poussière dore, près des pieds. Elle chatouille le pantalon. Elle est chaude. Tu t'assois, Amir ? Un peu. Une abeille visite une chaussure. Elle fait un petit bzz. Elle part. L'abeille a fini. L'herbe du parc sent le soleil. Ça sent l'herbe, maman. Tu la sens, l'herbe chaude ? Oui, maman. En ce moment, Amir prend la chaîne. Je veux jouer, maintenant ! Tout de suite ? Oui, papa. Les mains serrent le fer tiède. Tu pousses le siège ? Oui, maman. Nino arrive près de la balançoire. Il ouvre les bras trop vite. Un câlin ! Tu viens, Nino ? Oui. Nino serre Amir contre lui. Le câlin colle trop fort. Oh. Je te tiens. Amir sent sa poitrine coincée. Le sourire d'Amir disparaît. Dans sa poitrine, ça se bouscule. L'envie et la peur se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Nino, Amir ? Oui, papa. Tes mains sont chaudes, Amir ? Un peu, maman. L'éclat de balançoire tremble, puis tient. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,18 +1241,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.22</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>stop</t>
+          <t>éclat de balançoire</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>560</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1319,70 +1319,74 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=il_veut_jouer_maintenant; tempo=posé puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Le banc du parc est encore chaud.
-narrateur|Le bois sent le soleil.
-narrateur|L'herbe coupée sent fort.
-narrateur|Une chaîne de balançoire tinte.
-narrateur|Une feuille sèche tourne sur le chemin.
-narrateur|Un oiseau crie tout près, puis plus.
-maman|Je suis sur le banc, Victorina.
-maman|Tu joues près du bac à sable ?
-enfant-f|Oui, maman.
-narrateur|En ce moment, Victorina est près du bac.
-narrateur|Le sable est tiède sous les doigts.
-narrateur|Elle fait un petit tas, tout rond.
-maman|Je te vois, Victorina.
-maman|Le banc est juste ici.
-enfant-f|Mon tas est rond.
-maman|Il est bien rond, oui.
-narrateur|Chouchou arrive, tout content.
-narrateur|Il veut un câlin.
-narrateur|Le câlin est trop fort.
-narrateur|Victorina sent sa poitrine coincée.
-narrateur|Ses épaules montent.
-enfant-f|Je n'aime pas.
-enfant-f|C'est trop.
-enfant-f|Stop.
-narrateur|Elle recule d'un pas.
-narrateur|Elle peut s'éloigner.
-narrateur|Elle s'éloigne vers le banc.
-narrateur|Maman est l'adulte sur le banc.
-narrateur|Victorina va vers maman.
-enfant-f|C'était trop.
-maman|Je t'écoute.
-maman|Tu as dit stop.
-maman|Tu t'es éloignée.
-maman|Tu es venue vers moi.
-narrateur|Victorina pose sa main dans la main de maman.
-maman|Souffle un peu.
-narrateur|Victorina souffle.
-narrateur|Ses épaules descendent.
-maman|Dire stop, c'est permis.
-maman|On s'éloigne.
-maman|On va vers un adulte.
-enfant-f|Stop.
-enfant-f|Puis le banc.
-maman|Bravo, Victorina.
-maman|Tu as les épaules plus douces, maintenant ?
-enfant-f|Oui, maman.
-narrateur|Chouchou reste près du bac.
-narrateur|Il joue avec le sable.
-narrateur|Victorina reste près du banc.
-maman|Tu veux rester assise ici ?
-enfant-f|Oui.
-enfant-f|Près de toi.
-maman|On regarde la feuille, ensemble.
-narrateur|La feuille sèche a arrêté de tourner.
-narrateur|Le banc est chaud sous les jambes.
-enfant-f|Je me suis éloignée.
-maman|Oui.
-maman|Vers un adulte.
-maman|C'est le bon geste.</t>
+          <t>narrateur|La chaîne de la balançoire tinte au soleil.
+enfant-m|Elle tinte, papa.
+papa|Tu l'entends, la chaîne ?
+enfant-m|Oui, papa.
+narrateur|Le siège sent le caoutchouc chaud.
+maman|Il est chaud, Amir ?
+enfant-m|Un peu, maman.
+narrateur|Papa tapote le fer du siège.
+narrateur|Toc, toc, sur le métal.
+papa|Tu entends le fer, Amir ?
+enfant-m|Oui, il sonne.
+narrateur|Maman pose la main sur le siège.
+narrateur|Le caoutchouc est tiède, un peu rêche.
+narrateur|Sur le fer, un éclat de balançoire luit.
+enfant-m|Il brille, maman.
+maman|Tu le vois, sur le fer ?
+enfant-m|Oui, un petit point.
+papa|Le soleil le touche.
+narrateur|Un rayon glisse entre les chaînes.
+narrateur|La poussière dore, près des pieds.
+narrateur|Elle chatouille le pantalon.
+enfant-m|Elle est chaude.
+maman|Tu t'assois, Amir ?
+enfant-m|Un peu.
+narrateur|Une abeille visite une chaussure.
+narrateur|Elle fait un petit bzz.
+enfant-m|Elle part.
+papa|L'abeille a fini.
+narrateur|L'herbe du parc sent le soleil.
+enfant-m|Ça sent l'herbe, maman.
+maman|Tu la sens, l'herbe chaude ?
+enfant-m|Oui, maman.
+narrateur|En ce moment, Amir prend la chaîne.
+enfant-m|Je veux jouer, maintenant !
+papa|Tout de suite ?
+enfant-m|Oui, papa.
+narrateur|Les mains serrent le fer tiède.
+maman|Tu pousses le siège ?
+enfant-m|Oui, maman.
+narrateur|Nino arrive près de la balançoire.
+narrateur|Il ouvre les bras trop vite.
+copain|Un câlin !
+enfant-m|Tu viens, Nino ?
+copain|Oui.
+narrateur|Nino serre Amir contre lui.
+narrateur|Le câlin colle trop fort.
+enfant-m|Oh.
+copain|Je te tiens.
+narrateur|Amir sent sa poitrine coincée.
+narrateur|Le sourire d'Amir disparaît.
+narrateur|Dans sa poitrine, ça se bouscule.
+narrateur|L'envie et la peur se heurtent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Nino, Amir ?
+enfant-m|Oui, papa.
+maman|Tes mains sont chaudes, Amir ?
+enfant-m|Un peu, maman.
+narrateur|L'éclat de balançoire tremble, puis tient.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1414,17 +1418,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>C'est trop pour Victorina. Que dit-elle ?</t>
+          <t>C'est trop pour Amir. Que dit-il ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>C'est trop pour Victorina. Que dit-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;C'est trop pour &lt;emphasis level="moderate"&gt;Amir&lt;/emphasis&gt;. Que dit-il ?&lt;/prosody&gt;&lt;break time="780ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;C'est trop pour Adam. Que dit-il ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;C'est trop pour &lt;emphasis&gt;Amir&lt;/emphasis&gt;. Que dit-il ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1449,7 +1453,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Adam dit stop. Puis il va où ?</t>
+          <t>Amir dit stop. Puis il va où ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1487,7 +1491,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1498,7 +1502,7 @@
         <v>0.8</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.36</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1513,34 +1517,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Amir</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>780</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>360</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.3</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1555,7 +1563,7 @@
         <v>0.8</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1565,13 +1573,13 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=c_est_trop_pour_amir_que_dit_il; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|C'est trop pour Victorina.
-narrateur|Que dit-elle ?</t>
+          <t>narrateur|C'est trop pour Amir.
+narrateur|Que dit-il ?</t>
         </is>
       </c>
     </row>
@@ -1598,17 +1606,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Victorina a dit stop. Elle a pu s'éloigner. Elle rejoint maman, l'adulte. Stop, s'éloigner, un adulte. Bravo. J'ai dit stop. Je me suis éloignée. Oui. Vers moi, l'adulte.</t>
+          <t>Amir veut le siège, tout de suite. Je pousse, maintenant ! Nino serre trop, trop près. Les mots se bousculent dans sa bouche. Viens. Nino avance d'un pas. Stop. Amir recule d'un pas. Le sourire ne revient pas. Amir refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le siège, un instant. Il écoute la chaîne de la balançoire. Tu veux le siège avec Nino ? Papa reste à la même hauteur. Tu restes un peu loin ? Nino ne dit rien, d'abord. Il ouvre les bras, puis les baisse. Je m'arrête. D'accord. Merci, Amir. Papa a vu les deux, près du fer. La poussière colle un peu, sous les doigts. Elle est tiède. Amir essuie le siège du plat de la main. Nino reste un pas plus loin. Le siège avance sans coller, cette fois. Il bouge ! Oui. Tu le vois, le siège ? Oui, papa. Tu pousses, Nino ? J'y vais. Amir pousse, sans se presser. Nino suit le siège des yeux. Le siège danse une fois. Un. Deux. Le ventre d'Amir se desserre. Les épaules se relèvent un peu. On reste près de la balançoire ? Oui. Tes mains sont au chaud ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Victorina a dit stop. Elle a pu s'éloigner. Elle rejoint maman, l'adulte. Stop, s'éloigner, un adulte. Bravo. J'ai dit stop. Je me suis éloignée. Oui. Vers moi, l'adulte.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Amir veut le siège, tout de suite. Je pousse, maintenant ! Nino serre trop, trop près. Les mots se bousculent dans sa bouche. Viens. Nino avance d'un pas. Stop. Amir recule d'un pas. Le sourire ne revient pas. Amir refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le siège, un instant. Il écoute la chaîne de la balançoire. Tu veux le siège avec Nino ? Papa reste à la même hauteur. Tu restes un peu loin ? Nino ne dit rien, d'abord. Il ouvre les bras, puis les baisse. Je m'arrête. D'accord. Merci, Amir. Papa a vu les deux, près du fer. La poussière colle un peu, sous les doigts. Elle est tiède. Amir essuie le siège du plat de la main. Nino reste un pas plus loin. Le siège avance sans coller, cette fois. Il bouge ! Oui. Tu le vois, le siège ? Oui, papa. Tu pousses, Nino ? J'y vais. Amir pousse, sans se presser. Nino suit le siège des yeux. Le siège danse une fois. Un. Deux. Le ventre d'Amir se desserre. Les épaules se relèvent un peu. On reste près de la balançoire ? Oui. Tes mains sont au chaud ? Un peu, maman.&lt;/prosody&gt;&lt;break time="620ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Adam a dit &lt;emphasis&gt;stop&lt;/emphasis&gt;. Il a pu s'éloigner. Il rejoint maman, l'adulte.&lt;/slow&gt; [pause]</t>
+          <t>Amir veut le siège, tout de suite. Je pousse, maintenant ! Nino serre trop, trop près. Les mots se bousculent dans sa bouche. Viens. Nino avance d'un pas. Stop. Amir recule d'un pas. Le sourire ne revient pas. Amir refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le siège, un instant. Il écoute la chaîne de la balançoire. Tu veux le siège avec Nino ? Papa reste à la même hauteur. Tu restes un peu loin ? Nino ne dit rien, d'abord. Il ouvre les bras, puis les baisse. Je m'arrête. D'accord. Merci, Amir. Papa a vu les deux, près du fer. La poussière colle un peu, sous les doigts. Elle est tiède. Amir essuie le siège du plat de la main. Nino reste un pas plus loin. Le siège avance sans coller, cette fois. Il bouge ! Oui. Tu le vois, le siège ? Oui, papa. Tu pousses, Nino ? J'y vais. Amir pousse, sans se presser. Nino suit le siège des yeux. Le siège danse une fois. Un. Deux. Le ventre d'Amir se desserre. Les épaules se relèvent un peu. On reste près de la balançoire ? Oui. Tes mains sont au chaud ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1655,18 +1663,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.24</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1696,23 +1704,23 @@
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>620</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>310</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.33</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1721,10 +1729,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1733,24 +1741,65 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_dit_stop_il_recule; tempo=posé; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Victorina a dit stop.
-narrateur|Elle a pu s'éloigner.
-narrateur|Elle rejoint maman, l'adulte.
-maman|Stop, s'éloigner, un adulte.
-maman|Bravo.
-enfant-f|J'ai dit stop.
-enfant-f|Je me suis éloignée.
-maman|Oui.
-maman|Vers moi, l'adulte.</t>
+          <t>narrateur|Amir veut le siège, tout de suite.
+enfant-m|Je pousse, maintenant !
+narrateur|Nino serre trop, trop près.
+narrateur|Les mots se bousculent dans sa bouche.
+copain|Viens.
+narrateur|Nino avance d'un pas.
+enfant-m|Stop.
+narrateur|Amir recule d'un pas.
+narrateur|Le sourire ne revient pas.
+narrateur|Amir refuse de foncer.
+narrateur|Il referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Il observe le siège, un instant.
+narrateur|Il écoute la chaîne de la balançoire.
+papa|Tu veux le siège avec Nino ?
+narrateur|Papa reste à la même hauteur.
+enfant-m|Tu restes un peu loin ?
+narrateur|Nino ne dit rien, d'abord.
+narrateur|Il ouvre les bras, puis les baisse.
+copain|Je m'arrête.
+enfant-m|D'accord.
+papa|Merci, Amir.
+narrateur|Papa a vu les deux, près du fer.
+maman|La poussière colle un peu, sous les doigts.
+enfant-m|Elle est tiède.
+narrateur|Amir essuie le siège du plat de la main.
+narrateur|Nino reste un pas plus loin.
+narrateur|Le siège avance sans coller, cette fois.
+enfant-m|Il bouge !
+copain|Oui.
+papa|Tu le vois, le siège ?
+enfant-m|Oui, papa.
+maman|Tu pousses, Nino ?
+copain|J'y vais.
+narrateur|Amir pousse, sans se presser.
+narrateur|Nino suit le siège des yeux.
+narrateur|Le siège danse une fois.
+copain|Un.
+enfant-m|Deux.
+narrateur|Le ventre d'Amir se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|On reste près de la balançoire ?
+enfant-m|Oui.
+maman|Tes mains sont au chaud ?
+enfant-m|Un peu, maman.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>enfants_parc</t>
         </is>
       </c>
     </row>
@@ -1777,17 +1826,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Victorina reste près du banc. On reste ici un peu ? Oui. Je te parle tout bas. Ta main est dans ma main. Je me suis éloignée. Oui. Vers l'adulte. Tu as dit stop. La chaîne de balançoire tinte encore, loin. L'herbe sent toujours fort. Le tas de sable reste rond, là-bas.</t>
+          <t>Maman pose un seau près de l'herbe. Il est un peu poudreux. Le siège, maintenant ! Nino court trop, tout de suite. Il se colle trop près du siège. Avec moi ! Le siège penche vers Nino. Il penche ! Amir avance les mains, trop vite. Puis il s'arrête net. Amir refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le siège, un instant. Il écoute la chaîne de la balançoire. Sur le fer, un éclat de balançoire luit. Là, sur le fer. Stop. Amir recule d'un pas. Nino ne dit rien. Il souffle, puis recule aussi. Oui. On tient la chaîne ? Oui, papa. La chaîne sent le fer chaud. Le siège est là, un peu tiède. Amir le pousse vers Nino. Nino le rend, sans se coller. Poumf. Poumf. Le siège est bien calme ? Oui, papa. La poussière est chaude, Nino ? Un peu. Ils poussent le siège, à un pas. L'herbe chatouille les genoux. C'est plus facile. La balançoire est calme ? Oui, papa. Un rayon passe entre les chaînes. Il allume le fer.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Victorina reste près du banc. On reste ici un peu ? Oui. Je te parle tout bas. Ta main est dans ma main. Je me suis éloignée. Oui. Vers l'adulte. Tu as dit stop. La chaîne de balançoire tinte encore, loin. L'herbe sent toujours fort. Le tas de sable reste rond, là-bas.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman pose un seau près de l'herbe. Il est un peu poudreux. Le siège, maintenant ! Nino court trop, tout de suite. Il se colle trop près du siège. Avec moi ! Le siège penche vers Nino. Il penche ! Amir avance les mains, trop vite. Puis il s'arrête net. Amir refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le siège, un instant. Il écoute la chaîne de la balançoire. Sur le fer, un &lt;emphasis level="moderate"&gt;éclat de balançoire&lt;/emphasis&gt; luit. Là, sur le fer. Stop. Amir recule d'un pas. Nino ne dit rien. Il souffle, puis recule aussi. Oui. On tient la chaîne ? Oui, papa. La chaîne sent le fer chaud. Le siège est là, un peu tiède. Amir le pousse vers Nino. Nino le rend, sans se coller. Poumf. Poumf. Le siège est bien calme ? Oui, papa. La poussière est chaude, Nino ? Un peu. Ils poussent le siège, à un pas. L'herbe chatouille les genoux. C'est plus facile. La balançoire est calme ? Oui, papa. Un rayon passe entre les chaînes. Il allume le fer.&lt;/prosody&gt;&lt;break time="480ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Adam reste près du banc. Maman lui parle tout bas.&lt;/slow&gt; [pause]</t>
+          <t>Maman pose un seau près de l'herbe. Il est un peu poudreux. Le siège, maintenant ! Nino court trop, tout de suite. Il se colle trop près du siège. Avec moi ! Le siège penche vers Nino. Il penche ! Amir avance les mains, trop vite. Puis il s'arrête net. Amir refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le siège, un instant. Il écoute la chaîne de la balançoire. Sur le fer, un &lt;emphasis&gt;éclat de balançoire&lt;/emphasis&gt; luit. Là, sur le fer. Stop. Amir recule d'un pas. Nino ne dit rien. Il souffle, puis recule aussi. Oui. On tient la chaîne ? Oui, papa. La chaîne sent le fer chaud. Le siège est là, un peu tiède. Amir le pousse vers Nino. Nino le rend, sans se coller. Poumf. Poumf. Le siège est bien calme ? Oui, papa. La poussière est chaude, Nino ? Un peu. Ils poussent le siège, à un pas. L'herbe chatouille les genoux. C'est plus facile. La balançoire est calme ? Oui, papa. Un rayon passe entre les chaînes. Il allume le fer. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1834,18 +1883,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1866,28 +1915,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de balançoire</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>480</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>280</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1896,10 +1949,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1908,23 +1961,61 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=nino_trop_pres_du_siege_il_s_arrete; tempo=un peu vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Victorina reste près du banc.
-maman|On reste ici un peu ?
-enfant-f|Oui.
-maman|Je te parle tout bas.
-maman|Ta main est dans ma main.
-enfant-f|Je me suis éloignée.
-maman|Oui.
-maman|Vers l'adulte.
-maman|Tu as dit stop.
-narrateur|La chaîne de balançoire tinte encore, loin.
-narrateur|L'herbe sent toujours fort.
-narrateur|Le tas de sable reste rond, là-bas.</t>
+          <t>narrateur|Maman pose un seau près de l'herbe.
+narrateur|Il est un peu poudreux.
+enfant-m|Le siège, maintenant !
+narrateur|Nino court trop, tout de suite.
+narrateur|Il se colle trop près du siège.
+copain|Avec moi !
+narrateur|Le siège penche vers Nino.
+enfant-m|Il penche !
+narrateur|Amir avance les mains, trop vite.
+narrateur|Puis il s'arrête net.
+narrateur|Amir refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Il observe le siège, un instant.
+narrateur|Il écoute la chaîne de la balançoire.
+narrateur|Sur le fer, un éclat de balançoire luit.
+enfant-m|Là, sur le fer.
+enfant-m|Stop.
+narrateur|Amir recule d'un pas.
+narrateur|Nino ne dit rien.
+narrateur|Il souffle, puis recule aussi.
+copain|Oui.
+papa|On tient la chaîne ?
+enfant-m|Oui, papa.
+narrateur|La chaîne sent le fer chaud.
+narrateur|Le siège est là, un peu tiède.
+narrateur|Amir le pousse vers Nino.
+narrateur|Nino le rend, sans se coller.
+enfant-m|Poumf.
+copain|Poumf.
+papa|Le siège est bien calme ?
+enfant-m|Oui, papa.
+maman|La poussière est chaude, Nino ?
+copain|Un peu.
+narrateur|Ils poussent le siège, à un pas.
+narrateur|L'herbe chatouille les genoux.
+enfant-m|C'est plus facile.
+papa|La balançoire est calme ?
+enfant-m|Oui, papa.
+maman|Un rayon passe entre les chaînes.
+enfant-m|Il allume le fer.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>enfants_parc</t>
         </is>
       </c>
     </row>
@@ -1951,17 +2042,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit stop. Je suis allée vers maman. Bravo. Le banc est encore un peu chaud.</t>
+          <t>Ils restent près de la chaîne. Maman essuie un peu de poussière. Le siège a penché, papa. Tu l'as vu, toi ? Oui, près de la balançoire. On est bien, ici. Amir tapote le fer du doigt. Il a une trace de poussière. Tu la vois, la trace ? Oui, maman. Le siège est resté, Amir. Oui, avec Nino. Le siège est resté. Ça sent le caoutchouc, un peu tiède. Et le fer, maman. Oui, dans l'air. Le siège reste près de l'herbe. Un éclat de balançoire tient sur le fer.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit stop. Je suis allée vers maman. Bravo. Le banc est encore un peu chaud.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la chaîne. Maman essuie un peu de poussière. Le siège a penché, papa. Tu l'as vu, toi ? Oui, près de la balançoire. On est bien, ici. Amir tapote le fer du doigt. Il a une trace de poussière. Tu la vois, la trace ? Oui, maman. Le siège est resté, Amir. Oui, avec Nino. Le siège est resté. Ça sent le caoutchouc, un peu tiède. Et le fer, maman. Oui, dans l'air. Le siège reste près de l'herbe. Un &lt;emphasis level="moderate"&gt;éclat de balançoire&lt;/emphasis&gt; tient sur le fer.&lt;/prosody&gt;&lt;break time="980ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la chaîne. Maman essuie un peu de poussière. Le siège a penché, papa. Tu l'as vu, toi ? Oui, près de la balançoire. On est bien, ici. Amir tapote le fer du doigt. Il a une trace de poussière. Tu la vois, la trace ? Oui, maman. Le siège est resté, Amir. Oui, avec Nino. Le siège est resté. Ça sent le caoutchouc, un peu tiède. Et le fer, maman. Oui, dans l'air. Le siège reste près de l'herbe. Un &lt;emphasis&gt;éclat de balançoire&lt;/emphasis&gt; tient sur le fer.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2008,7 +2099,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2016,7 +2107,7 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AB6" s="2" t="n">
         <v>1.36</v>
@@ -2028,12 +2119,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2042,14 +2133,18 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de balançoire</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>980</v>
       </c>
       <c r="AK6" s="2" t="n">
         <v>380</v>
@@ -2061,11 +2156,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.29</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2074,27 +2169,45 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_fer; tempo=très posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai dit stop.
-enfant-f|Je suis allée vers maman.
-maman|Bravo.
-narrateur|Le banc est encore un peu chaud.</t>
+          <t>narrateur|Ils restent près de la chaîne.
+narrateur|Maman essuie un peu de poussière.
+enfant-m|Le siège a penché, papa.
+papa|Tu l'as vu, toi ?
+enfant-m|Oui, près de la balançoire.
+maman|On est bien, ici.
+narrateur|Amir tapote le fer du doigt.
+enfant-m|Il a une trace de poussière.
+maman|Tu la vois, la trace ?
+enfant-m|Oui, maman.
+papa|Le siège est resté, Amir.
+enfant-m|Oui, avec Nino.
+copain|Le siège est resté.
+narrateur|Ça sent le caoutchouc, un peu tiède.
+enfant-m|Et le fer, maman.
+maman|Oui, dans l'air.
+narrateur|Le siège reste près de l'herbe.
+narrateur|Un éclat de balançoire tient sur le fer.</t>
         </is>
       </c>
     </row>
@@ -2115,7 +2228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2179,6 +2292,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>